<commit_message>
extended login invalid cases
</commit_message>
<xml_diff>
--- a/testData/RegistrationData.xlsx
+++ b/testData/RegistrationData.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Email</t>
   </si>
@@ -96,6 +96,12 @@
   </si>
   <si>
     <t>Test@012</t>
+  </si>
+  <si>
+    <t>hlgox960@gmail.com</t>
+  </si>
+  <si>
+    <t>Test@648</t>
   </si>
 </sst>
 </file>
@@ -140,7 +146,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -255,6 +261,14 @@
         <v>27</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>